<commit_message>
progress: 22 village workbooks (sivaramans-llin 2026-10-09T10:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
@@ -2402,6 +2402,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2409,6 +2414,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2416,6 +2426,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2423,6 +2438,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 1A1A1, 1A1B, 1A1C, 1A1D, 1A2, 1A3, 1B1A, 1B1B, 1B2, 2A1A, 2A1B, 2A2, 2A3, 2B1A, 2B1B, 2B2, 2C1A, 2C1B, 2C2, 2D1, 2D2, 3A, 3B1, 3B2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2430,6 +2450,11 @@
           <t>258</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A1A2, 1A1A3, 1A1B, 1A2, 1B1, 1B2, 1C1, 1C2, 1D1, 1D2, 1E1, 1E2, 2A, 2B, 2C1A, 2C1B, 2C2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2437,6 +2462,11 @@
           <t>259</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2444,6 +2474,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2451,6 +2486,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2458,6 +2498,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B, 2C, 2D, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2465,6 +2510,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2472,6 +2522,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2479,6 +2534,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2486,6 +2546,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2493,6 +2558,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2500,6 +2570,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2507,6 +2582,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2514,6 +2594,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2521,6 +2606,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B, 3A, 3B1, 3B2, 3B3, 4A, 4B, 4C, 4D, 4E</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2528,6 +2618,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2535,6 +2630,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2542,6 +2642,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2549,6 +2654,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 4A, 4B, 4C, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2556,6 +2666,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2563,6 +2678,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2570,6 +2690,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2577,6 +2702,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2584,11 +2714,21 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
           <t>279</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 22 village workbooks (sivaramans-llin 2026-10-09T10:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
@@ -2738,6 +2738,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2745,6 +2750,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2C, 2D, 3A1A1A, 3A1A2, 3A2, 3A3, 3A4, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2752,6 +2762,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2759,6 +2774,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2766,6 +2786,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2773,6 +2798,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2780,6 +2810,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2787,6 +2822,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2794,6 +2834,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2801,6 +2846,11 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B, 2B2C, 3A1A, 3A1B, 3A2, 3A3A, 3A3B, 3B, 3C, 3D, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2808,6 +2858,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2815,6 +2870,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2822,6 +2882,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2829,6 +2894,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2836,6 +2906,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2843,6 +2918,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2850,6 +2930,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2857,6 +2942,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3A1A, 3A1B, 3A2, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2864,6 +2954,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2871,6 +2966,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2878,6 +2978,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2885,6 +2990,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 4C, 4D, 4E</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2892,6 +3002,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2899,6 +3014,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2906,6 +3026,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2913,6 +3038,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2920,6 +3050,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1A1, 2A1B, 2A1C, 2A2, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2927,6 +3062,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2934,6 +3074,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2941,6 +3086,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2948,6 +3098,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2955,6 +3110,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4B, 4C, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2962,6 +3122,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C, 3D1, 3D2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2969,6 +3134,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2976,6 +3146,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2983,6 +3158,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2990,6 +3170,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2997,6 +3182,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -3004,6 +3194,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -3011,6 +3206,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -3018,6 +3218,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3025,6 +3230,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3032,6 +3242,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3039,6 +3254,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1A, 1B</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3046,6 +3266,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3053,6 +3278,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3060,6 +3290,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B1, 2B2, 2B3, 3A, 3B, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3067,6 +3302,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3074,6 +3314,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3081,6 +3326,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3088,6 +3338,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3095,6 +3350,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3102,6 +3362,11 @@
           <t>326</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3109,6 +3374,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3116,6 +3386,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3123,6 +3398,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3, 4, 5A, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3130,6 +3410,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3137,6 +3422,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3144,6 +3434,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D1, 2D2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3151,6 +3446,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3158,6 +3458,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3165,6 +3470,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3172,6 +3482,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3179,6 +3494,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3186,6 +3506,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3193,6 +3518,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3200,11 +3530,21 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
           <t>34</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 22 village workbooks (sivaramans-llin 2026-10-09T10:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
@@ -3554,6 +3554,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 3</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3561,6 +3566,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11, 1A1, 1A2, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3568,6 +3578,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3575,6 +3590,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3582,6 +3602,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3589,6 +3614,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3596,6 +3626,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3603,6 +3638,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3610,6 +3650,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3617,6 +3662,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3624,6 +3674,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3631,6 +3686,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3638,6 +3698,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3645,6 +3710,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3652,6 +3722,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3659,6 +3734,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3666,6 +3746,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3673,6 +3758,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3680,6 +3770,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3687,6 +3782,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3694,6 +3794,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1A, 2A1B, 2A2, 2A3, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3701,6 +3806,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5, 6A, 6B1, 6B2, 6B3, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3708,6 +3818,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3715,6 +3830,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3722,6 +3842,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3729,6 +3854,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3736,6 +3866,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1A, 1A1, 1A2, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3743,6 +3878,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3750,6 +3890,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3757,6 +3902,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1O, 1P, 1Q1, 1Q2, 1R, 1S, 1T, 1U, 2</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3764,6 +3914,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3771,6 +3926,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1B4A, 1B4B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3778,6 +3938,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3785,6 +3950,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B1A, 1B1B, 1B2, 1B3, 1B4, 1C1A, 1C1B, 1C2, 1D, 1E, 2A, 2B, 2C, 2D, 3, 4A1, 4A2, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3792,6 +3962,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2A3, 2B1, 2B2, 2C1A, 2C1B, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3799,6 +3974,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3806,6 +3986,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A1A, 3A1B, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3813,6 +3998,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3820,6 +4010,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3A, 1A3B, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3827,6 +4022,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3834,6 +4034,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3841,6 +4046,11 @@
           <t>379</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3848,6 +4058,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3855,6 +4070,11 @@
           <t>380</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3862,6 +4082,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B1A, 2B1B, 2B1C, 2B2, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3869,6 +4094,11 @@
           <t>382</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3876,6 +4106,11 @@
           <t>383</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3883,6 +4118,11 @@
           <t>384</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3890,6 +4130,11 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -3897,6 +4142,11 @@
           <t>386</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -3904,6 +4154,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F1, 1F2, 1G, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -3911,6 +4166,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -3918,6 +4178,11 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -3925,6 +4190,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A2, 1A3, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -3932,6 +4202,11 @@
           <t>394</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1A2, 1A1B, 1A2, 1A3, 1A4, 1B, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -3939,6 +4214,11 @@
           <t>395</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>1, 2A1A1, 2A2, 2A3, 2A4, 2B, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -3946,6 +4226,11 @@
           <t>396</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C1A, 3C1B, 3C2, 3C3A, 3C3B, 3C3C</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -3953,6 +4238,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A1, 3A2, 3B, 3C1, 3C2</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -3960,6 +4250,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -3967,6 +4262,11 @@
           <t>399</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -3974,6 +4274,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B1, 3B2, 3B3, 3B4, 3B5, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -3981,6 +4286,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -3988,6 +4298,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -3995,6 +4310,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4002,6 +4322,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4009,6 +4334,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1C, 1D1, 1D2, 1E, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4016,6 +4346,11 @@
           <t>404</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 3</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4023,6 +4358,11 @@
           <t>405</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4030,6 +4370,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4037,6 +4382,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B1, 2B2, 2C, 2D, 2E1, 2E1A2, 2E1B, 2E2, 2E3, 2F, 2G, 2H, 3, 4, 5A, 5B, 6A, 6B1, 6B2, 6C, 7A, 7B, 7C, 7D, 8A, 8B1, 8B2, 8C1, 8C2, 8D1, 8D2, 8E, 8F, 9</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4044,6 +4394,11 @@
           <t>408</t>
         </is>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1, 1C2, 1C3, 1C4, 1D1, 1D2, 1D3, 1D4, 1D5, 1D6, 1E, 1F, 2</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4051,6 +4406,11 @@
           <t>409</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D1A, 1D2, 1D3, 1D4, 1D5, 1D6, 1D7, 2A, 2B, 3A, 3B, 3C, 4A1, 4A2, 4B, 4C1, 4C2, 4D1A, 4D2, 4D3, 4E1, 4E2, 4E3, 5A, 5B, 5C, 5D, 5E, 6</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4058,6 +4418,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2A, 2B, 2C, 3A, 3B, 3C, 4A, 4B, 4C, 4D, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4065,6 +4430,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4072,6 +4442,11 @@
           <t>411</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4079,6 +4454,11 @@
           <t>412</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4086,6 +4466,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 10F, 2A, 2B, 2C, 2D, 3, 4A, 4B, 5A, 5B, 5C1, 5C2, 6A, 6B, 6C, 6D, 6E, 6F, 7A, 7B, 8A, 8B, 8C, 8D, 8E, 8F, 8G, 8H, 8I1, 8I2, 8I3, 8J1, 8J2, 8K1A, 8K1B, 8K2, 8K3, 8L1, 8L2, 8L3, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4093,6 +4478,11 @@
           <t>414</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4100,6 +4490,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4107,6 +4502,11 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16A, 16B, 16C, 17, 18, 19, 2, 20, 21, 22, 23, 24A, 24B, 25, 26, 27, 28, 29A1A1A, 29A2, 29A3A, 29A3B, 29A4, 29B, 29C, 3, 30, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4114,6 +4514,11 @@
           <t>417</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B1, 2B2, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4121,6 +4526,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4128,11 +4538,21 @@
           <t>419</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
           <t>42</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 22 village workbooks (sivaramans-llin 2026-10-09T10:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
@@ -4562,6 +4562,11 @@
           <t>420</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4569,6 +4574,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4576,6 +4586,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4583,6 +4598,11 @@
           <t>423</t>
         </is>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4590,6 +4610,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4597,6 +4622,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4604,6 +4634,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4611,6 +4646,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4618,6 +4658,11 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4625,6 +4670,11 @@
           <t>429</t>
         </is>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4632,6 +4682,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4639,6 +4694,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4646,6 +4706,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 3A, 3B, 4, 5A1, 5A2, 5A3, 5A4, 5A5, 5A6, 5A7, 5A8, 5A9, 5B, 5C, 6A, 6B, 6C, 7, 8, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4653,6 +4718,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A1, 5A2, 5A3, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4660,6 +4730,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 2A1A, 2A1B, 2A1C, 2A1D, 2A2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4667,6 +4742,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4674,6 +4754,11 @@
           <t>435</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4681,6 +4766,11 @@
           <t>436</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4688,6 +4778,11 @@
           <t>437</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4695,6 +4790,11 @@
           <t>438</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A1, 3A2, 3B1, 3B2, 3B3, 3C1A, 3C1B, 3C2, 3D1, 3D2, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4702,6 +4802,11 @@
           <t>439</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4709,6 +4814,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 2, 3, 4, 5, 6A, 6B, 7A1, 7A2, 7B1, 7B2, 7C1, 7C2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4716,6 +4826,11 @@
           <t>440</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4723,6 +4838,11 @@
           <t>441</t>
         </is>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1A, 1B</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4730,6 +4850,11 @@
           <t>442</t>
         </is>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4737,6 +4862,11 @@
           <t>443</t>
         </is>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4744,6 +4874,11 @@
           <t>444</t>
         </is>
       </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C1A, 6C2, 6C3A, 6C3B</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4751,6 +4886,11 @@
           <t>445</t>
         </is>
       </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4758,6 +4898,11 @@
           <t>446</t>
         </is>
       </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4765,6 +4910,11 @@
           <t>447</t>
         </is>
       </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>1A1, 1A1B, 1A2, 1A3, 1B, 2, 3A, 3B, 3C1, 3C2, 3C3, 3C4, 4</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4772,6 +4922,11 @@
           <t>448</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4779,6 +4934,11 @@
           <t>449</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4A2, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4786,6 +4946,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4793,6 +4958,11 @@
           <t>450</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1A1, 3A1A2, 3A2, 3A3, 3B, 4A1, 4A2, 4A3, 4A4, 4A5, 4B, 5A, 5B1, 5B2, 5B3, 5B4, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4800,6 +4970,11 @@
           <t>451</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4807,6 +4982,11 @@
           <t>452</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4814,6 +4994,11 @@
           <t>453</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 1A1, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4821,6 +5006,11 @@
           <t>454</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4828,6 +5018,11 @@
           <t>455</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4835,6 +5030,11 @@
           <t>456</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4842,6 +5042,11 @@
           <t>457</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4849,6 +5054,11 @@
           <t>458</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -4856,6 +5066,11 @@
           <t>459</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -4863,6 +5078,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -4870,6 +5090,11 @@
           <t>460</t>
         </is>
       </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>10, 11, 1A2A, 1A2B, 1A3, 1B, 2, 3, 4, 4A1, 5, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -4877,6 +5102,11 @@
           <t>461</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -4884,6 +5114,11 @@
           <t>462</t>
         </is>
       </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11A, 11B, 11C, 11D, 12A, 12B, 12C, 13, 14A, 14B, 15, 16, 1A, 1B, 1C, 1D, 2, 3, 4A, 4B, 5, 6, 7A, 7B, 7C, 7D, 7E, 7F, 8A, 8B, 8C, 8D, 8E, 9</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -4891,6 +5126,11 @@
           <t>463</t>
         </is>
       </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -4898,6 +5138,11 @@
           <t>464</t>
         </is>
       </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -4905,6 +5150,11 @@
           <t>465</t>
         </is>
       </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -4912,6 +5162,11 @@
           <t>466</t>
         </is>
       </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 4A, 4B, 4C, 4D, 4E, 4F, 4G</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -4919,6 +5174,11 @@
           <t>467</t>
         </is>
       </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A2, 1A3, 1A4, 1B, 1C, 1D, 1E, 1F1, 1F2, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -4926,6 +5186,11 @@
           <t>468</t>
         </is>
       </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1B4, 1B5, 1B6, 1B7, 1B8, 1B9, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -4933,6 +5198,11 @@
           <t>469</t>
         </is>
       </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -4940,6 +5210,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>10, 1A1, 1A2, 1B1, 1B2, 1C1, 1C2, 2, 3A, 3B, 4, 5A, 5B, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -4947,6 +5222,11 @@
           <t>470</t>
         </is>
       </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -4954,6 +5234,11 @@
           <t>471</t>
         </is>
       </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -4961,6 +5246,11 @@
           <t>472</t>
         </is>
       </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -4968,6 +5258,11 @@
           <t>473</t>
         </is>
       </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -4975,6 +5270,11 @@
           <t>474</t>
         </is>
       </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -4982,6 +5282,11 @@
           <t>475</t>
         </is>
       </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -4989,6 +5294,11 @@
           <t>476</t>
         </is>
       </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -4996,6 +5306,11 @@
           <t>477</t>
         </is>
       </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 1C, 2A1, 2A2, 2B, 3, 4, 5, 6A, 6B, 6C, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -5003,6 +5318,11 @@
           <t>478</t>
         </is>
       </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -5010,6 +5330,11 @@
           <t>479</t>
         </is>
       </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -5017,6 +5342,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -5024,11 +5354,21 @@
           <t>480</t>
         </is>
       </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 4C, 5A1, 5A2, 5B, 5C, 6, 7, 8A, 8B, 8C, 8D, 9A, 9B, 9C, 9D, 9E</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
           <t>481</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1B, 1C</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 23 village workbooks (rw-rtx-3070 2026-10-09T14:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Natham_13.453312_80.144417.xlsx
@@ -5978,6 +5978,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -5985,6 +5990,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -5992,6 +6002,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -5999,6 +6014,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 2, 3, 4A, 4B, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -6006,6 +6026,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -6013,6 +6038,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3A, 3B, 3C, 3D1, 3D2</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -6020,6 +6050,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -6027,6 +6062,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -6034,6 +6074,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -6041,6 +6086,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -6048,6 +6098,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -6055,6 +6110,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -6062,6 +6122,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3, 4A, 4B1, 4B2, 4B3</t>
+        </is>
+      </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -6069,6 +6134,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -6076,6 +6146,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -6083,6 +6158,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -6090,6 +6170,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 12C, 1A, 1B, 2, 3A, 3B, 4, 5A, 5B, 5C, 5D, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -6097,6 +6182,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3A, 3B, 3C, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -6104,6 +6194,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>1A1, 1B, 2A, 2B, 3, 4A, 4B, 5A, 5B, 5C1, 5C2, 5C3</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -6111,6 +6206,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -6118,6 +6218,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -6125,6 +6230,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -6132,6 +6242,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -6139,6 +6254,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -6146,6 +6266,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -6153,6 +6278,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -6160,6 +6290,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -6167,11 +6302,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2A, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6A1A, 6A1B, 6A2, 6B, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>